<commit_message>
Actualizado al 11 Agosto 2025
</commit_message>
<xml_diff>
--- a/archivos/ALTAS.xlsx
+++ b/archivos/ALTAS.xlsx
@@ -8,19 +8,19 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja5" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t xml:space="preserve">Apellido</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Sexo</t>
   </si>
   <si>
-    <t xml:space="preserve">C- Postal</t>
+    <t xml:space="preserve">CP</t>
   </si>
   <si>
     <t xml:space="preserve">Tel Caract.</t>
@@ -76,69 +76,156 @@
     <t xml:space="preserve">CUIT/CUIL</t>
   </si>
   <si>
-    <t xml:space="preserve">Candia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mariel Gisella</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nicolas Tarifa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allen</t>
+    <t xml:space="preserve">COMAMALA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VANINA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P. nacional Iguazu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bariloche</t>
   </si>
   <si>
     <t xml:space="preserve">F</t>
   </si>
   <si>
-    <t xml:space="preserve">S</t>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06021975</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PALACIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCELA YOLANDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14071967</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAL BIANCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARIA ALEXA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con Con</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05041974</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="d&quot; de &quot;mmmm"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="5">
-    <font>
+  <fonts count="13">
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000009"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000009"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -182,24 +269,64 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -212,6 +339,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF000009"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF222222"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -326,10 +513,27 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="13.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="5.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="6.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="8.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="8.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="9.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="13.81"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -392,59 +596,165 @@
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1241</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2" t="s">
+      <c r="D2" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>8328</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>298</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>4382290</v>
-      </c>
-      <c r="M2" s="3" t="s">
+      <c r="J2" s="4" t="n">
+        <v>8400</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>2944</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>626184</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="4" t="n">
-        <v>24121988</v>
-      </c>
-      <c r="O2" s="2" t="n">
+      <c r="N2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="P2" s="2" t="n">
-        <v>34667675</v>
-      </c>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2" t="n">
-        <v>27346676758</v>
+      <c r="P2" s="4" t="n">
+        <v>24318207</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>27243182072</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>45924</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>432</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>8400</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>2944</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>665955</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>18493541</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>23184935414</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>7054</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>8400</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>2944</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>617289</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P4" s="14" t="n">
+        <v>23831193</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>23238311934</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>